<commit_message>
UK daily ratings for 2026-04-29
</commit_message>
<xml_diff>
--- a/output/daily_ratings/uk_ratings_2026-04-29.xlsx
+++ b/output/daily_ratings/uk_ratings_2026-04-29.xlsx
@@ -1898,17 +1898,17 @@
       </c>
       <c r="H25" t="inlineStr">
         <is>
-          <t>Racing Demon</t>
+          <t>Crafter (IRE)</t>
         </is>
       </c>
       <c r="I25" t="n">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="J25" t="n">
-        <v>134</v>
+        <v>130</v>
       </c>
       <c r="K25" t="n">
-        <v>59</v>
+        <v>55</v>
       </c>
       <c r="L25" t="inlineStr"/>
       <c r="M25" t="n">
@@ -1954,17 +1954,17 @@
       </c>
       <c r="H26" t="inlineStr">
         <is>
-          <t>Crafter (IRE)</t>
+          <t>Racing Demon</t>
         </is>
       </c>
       <c r="I26" t="n">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="J26" t="n">
-        <v>130</v>
+        <v>134</v>
       </c>
       <c r="K26" t="n">
-        <v>55</v>
+        <v>59</v>
       </c>
       <c r="L26" t="inlineStr"/>
       <c r="M26" t="n">
@@ -6478,17 +6478,17 @@
       </c>
       <c r="H102" t="inlineStr">
         <is>
-          <t>Pallas Lord (IRE)</t>
+          <t>Staffordshire (IRE)</t>
         </is>
       </c>
       <c r="I102" t="n">
-        <v>8</v>
+        <v>4</v>
       </c>
       <c r="J102" t="n">
-        <v>134</v>
+        <v>132</v>
       </c>
       <c r="K102" t="n">
-        <v>59</v>
+        <v>57</v>
       </c>
       <c r="L102" t="inlineStr"/>
       <c r="M102" t="n">
@@ -6534,17 +6534,17 @@
       </c>
       <c r="H103" t="inlineStr">
         <is>
-          <t>Staffordshire (IRE)</t>
+          <t>Pallas Lord (IRE)</t>
         </is>
       </c>
       <c r="I103" t="n">
-        <v>4</v>
+        <v>8</v>
       </c>
       <c r="J103" t="n">
-        <v>132</v>
+        <v>134</v>
       </c>
       <c r="K103" t="n">
-        <v>57</v>
+        <v>59</v>
       </c>
       <c r="L103" t="inlineStr"/>
       <c r="M103" t="n">

</xml_diff>